<commit_message>
Updating IVIS, survival and Cell Count analyses with latest results of April 8, 2026
</commit_message>
<xml_diff>
--- a/StatisticalAnalyses/Raji/output/CellCountTests_CD19_Raji_M5vsWT.xlsx
+++ b/StatisticalAnalyses/Raji/output/CellCountTests_CD19_Raji_M5vsWT.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -394,7 +394,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.017</t>
+          <t>0.005</t>
         </is>
       </c>
     </row>
@@ -417,6 +417,116 @@
       <c r="D3" t="inlineStr">
         <is>
           <t>&lt;0.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>E97</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CD19</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0.53</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>E97</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CD19</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0.971</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>E103</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CD19</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>E103</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CD19</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>&lt;0.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>E103</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CD19</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0.211</t>
         </is>
       </c>
     </row>

</xml_diff>